<commit_message>
Jenna package refresh: 21 platforms (Books) + games content-map
- Coverage Excel/MD now list Books (#21): buy/listen/Libby + content-map retail proxies
- Note gametool_content (games -> content-map) companion resolver
- Refresh Jenna how-to with a Books section + book-franchise SEASON=Book N
- Track StreamScout-HowTo-Jenna.md in-repo so it ships with the package
- No-login count 16 of 21

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/streamscout/StreamScout-Platforms.xlsx
+++ b/streamscout/StreamScout-Platforms.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -110,6 +110,12 @@
       <b val="1"/>
       <color rgb="000A3D91"/>
       <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+      <color rgb="009AA7B4"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Aptos"/>
@@ -212,7 +218,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -277,13 +283,16 @@
     <xf numFmtId="0" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
@@ -651,7 +660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4.5" customWidth="1" min="1" max="1"/>
@@ -673,7 +682,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  One tool → every watch / play id  ·  20 platforms  ·  movies, series, podcasts &amp; audiobooks</t>
+          <t xml:space="preserve">  One tool → every watch / play id  ·  21 platforms  ·  movies, series, podcasts, audiobooks &amp; books</t>
         </is>
       </c>
     </row>
@@ -1454,78 +1463,139 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="26" customHeight="1">
-      <c r="A29" s="22" t="inlineStr">
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>📖  Books  ·  1   (buy · listen · library — feeds the content map)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="21" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Books</t>
+        </is>
+      </c>
+      <c r="C29" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D29" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>No login</t>
+        </is>
+      </c>
+      <c r="F29" s="11" t="inlineStr">
+        <is>
+          <t>buy + listen + library links</t>
+        </is>
+      </c>
+      <c r="G29" s="12" t="inlineStr">
+        <is>
+          <t>Whole franchise → ONE show, SEASON = Book N. Amazon Kindle/Print/Audio, Audible, Apple Books, Libby holds, + retail proxies (Target/BAM, Walmart, B&amp;N, Bookshop, Costco). Feeds the CONTENT map (punctuation kept).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="26" customHeight="1">
+      <c r="A31" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  Good to know</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="23" t="inlineStr">
-        <is>
-          <t>•  15 of 20 platforms need NO login. Only 5 need anything: Netflix &amp; HBO Max (browser login), Spotify (free API key), and Disney+ &amp; SiriusXM (situational).</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="24" t="inlineStr">
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="24" t="inlineStr">
+        <is>
+          <t>•  16 of 21 platforms need NO login. Only 5 need anything: Netflix &amp; HBO Max (browser login), Spotify (free API key), and Disney+ &amp; SiriusXM (situational).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="25" t="inlineStr">
         <is>
           <t>•  Access legend:  No login = anonymous  ·  Browser login = a Firefox/Chromium window drives itself  ·  Free API key = Spotify Client ID+Secret  ·  Situational = usually none, occasional login.</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="23" t="inlineStr">
-        <is>
-          <t>•  Every run writes one CSV to your Desktop:  SHOW · URL · PRODUCTION · PLATFORM · SEASON.  PRODUCTION (studio) fills in automatically; SEASON is blank for movies, podcasts, audiobooks, Apple TV+, BritBox &amp; YouTube.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="24" t="inlineStr">
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="24" t="inlineStr">
+        <is>
+          <t>•  Every run writes one CSV to your Desktop:  SHOW · URL · PRODUCTION · PLATFORM · SEASON.  PRODUCTION (studio) fills in automatically; SEASON is blank for movies, podcasts &amp; audiobooks (and Apple TV+, BritBox &amp; YouTube), and carries Book N for a book franchise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="25" t="inlineStr">
+        <is>
+          <t>•  Books resolves a whole franchise to ONE show: purchase (Amazon Kindle/Print, Bookshop, Costco…), audiobook (Audible, Apple, Amazon), and LIBRARY holds (Libby/OverDrive) — with content-map retail proxies for the bot-walled stores. Its URLs feed the CONTENT map, so slugs keep their punctuation (p/merciless-saints).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="24" t="inlineStr">
+        <is>
+          <t>•  Companion resolver: gametool_content (in streamscout/gametool_content) does the same job for VIDEO GAMES — every buy/play URL across 19 stores, also as content-map terms. Its sibling gametool_hostmap emits the punctuation-stripped hostmap form for a different pipeline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="25" t="inlineStr">
         <is>
           <t>•  Podcast platforms return one row per episode. Streaming platforms handle both movies and series, with flexible season picks (all · 1-3 · 1,4,6).</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="23" t="inlineStr">
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="24" t="inlineStr">
         <is>
           <t>•  SiriusXM title search is Netflix-style: one device code the first time on a new computer, then automatic. Pasting a SiriusXM show link never needs a login.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="24" t="inlineStr">
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="25" t="inlineStr">
         <is>
           <t>•  Audible returns TWO rows per audiobook — the direct audible.com/pd listen link AND the parallel amazon.com/dp 'Audible Audio Edition' (a different ASIN) — each labeled Audible / Amazon in the PLATFORM column.</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="23" t="inlineStr">
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="24" t="inlineStr">
         <is>
           <t>•  Amazon captures every clickstream form — all offer ASINs, the GTI in both encodings, shells + episodes, every film edition, and Amazon Channels (Lionsgate+, Starz…).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="17">
     <mergeCell ref="A32:G32"/>
     <mergeCell ref="A36:G36"/>
     <mergeCell ref="A33:G33"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A40:G40"/>
     <mergeCell ref="A31:G31"/>
     <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A39:G39"/>
     <mergeCell ref="A34:G34"/>
     <mergeCell ref="A35:G35"/>
     <mergeCell ref="A26:G26"/>
-    <mergeCell ref="A30:G30"/>
+    <mergeCell ref="A38:G38"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A28:G28"/>
     <mergeCell ref="A19:G19"/>
     <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A37:G37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Jenna package refresh: 21 platforms (Books) + games content-map (#191)
- Coverage Excel/MD now list Books (#21): buy/listen/Libby + content-map retail proxies
- Note gametool_content (games -> content-map) companion resolver
- Refresh Jenna how-to with a Books section + book-franchise SEASON=Book N
- Track StreamScout-HowTo-Jenna.md in-repo so it ships with the package
- No-login count 16 of 21

Co-authored-by: Jessie <jessie@Trina-McGillicutty.local>
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/streamscout/StreamScout-Platforms.xlsx
+++ b/streamscout/StreamScout-Platforms.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -110,6 +110,12 @@
       <b val="1"/>
       <color rgb="000A3D91"/>
       <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+      <color rgb="009AA7B4"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Aptos"/>
@@ -212,7 +218,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -277,13 +283,16 @@
     <xf numFmtId="0" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
@@ -651,7 +660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4.5" customWidth="1" min="1" max="1"/>
@@ -673,7 +682,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  One tool → every watch / play id  ·  20 platforms  ·  movies, series, podcasts &amp; audiobooks</t>
+          <t xml:space="preserve">  One tool → every watch / play id  ·  21 platforms  ·  movies, series, podcasts, audiobooks &amp; books</t>
         </is>
       </c>
     </row>
@@ -1454,78 +1463,139 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="26" customHeight="1">
-      <c r="A29" s="22" t="inlineStr">
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>📖  Books  ·  1   (buy · listen · library — feeds the content map)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="21" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Books</t>
+        </is>
+      </c>
+      <c r="C29" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D29" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>No login</t>
+        </is>
+      </c>
+      <c r="F29" s="11" t="inlineStr">
+        <is>
+          <t>buy + listen + library links</t>
+        </is>
+      </c>
+      <c r="G29" s="12" t="inlineStr">
+        <is>
+          <t>Whole franchise → ONE show, SEASON = Book N. Amazon Kindle/Print/Audio, Audible, Apple Books, Libby holds, + retail proxies (Target/BAM, Walmart, B&amp;N, Bookshop, Costco). Feeds the CONTENT map (punctuation kept).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="26" customHeight="1">
+      <c r="A31" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  Good to know</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="23" t="inlineStr">
-        <is>
-          <t>•  15 of 20 platforms need NO login. Only 5 need anything: Netflix &amp; HBO Max (browser login), Spotify (free API key), and Disney+ &amp; SiriusXM (situational).</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="24" t="inlineStr">
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="24" t="inlineStr">
+        <is>
+          <t>•  16 of 21 platforms need NO login. Only 5 need anything: Netflix &amp; HBO Max (browser login), Spotify (free API key), and Disney+ &amp; SiriusXM (situational).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="25" t="inlineStr">
         <is>
           <t>•  Access legend:  No login = anonymous  ·  Browser login = a Firefox/Chromium window drives itself  ·  Free API key = Spotify Client ID+Secret  ·  Situational = usually none, occasional login.</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="23" t="inlineStr">
-        <is>
-          <t>•  Every run writes one CSV to your Desktop:  SHOW · URL · PRODUCTION · PLATFORM · SEASON.  PRODUCTION (studio) fills in automatically; SEASON is blank for movies, podcasts, audiobooks, Apple TV+, BritBox &amp; YouTube.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="24" t="inlineStr">
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="24" t="inlineStr">
+        <is>
+          <t>•  Every run writes one CSV to your Desktop:  SHOW · URL · PRODUCTION · PLATFORM · SEASON.  PRODUCTION (studio) fills in automatically; SEASON is blank for movies, podcasts &amp; audiobooks (and Apple TV+, BritBox &amp; YouTube), and carries Book N for a book franchise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="25" t="inlineStr">
+        <is>
+          <t>•  Books resolves a whole franchise to ONE show: purchase (Amazon Kindle/Print, Bookshop, Costco…), audiobook (Audible, Apple, Amazon), and LIBRARY holds (Libby/OverDrive) — with content-map retail proxies for the bot-walled stores. Its URLs feed the CONTENT map, so slugs keep their punctuation (p/merciless-saints).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="24" t="inlineStr">
+        <is>
+          <t>•  Companion resolver: gametool_content (in streamscout/gametool_content) does the same job for VIDEO GAMES — every buy/play URL across 19 stores, also as content-map terms. Its sibling gametool_hostmap emits the punctuation-stripped hostmap form for a different pipeline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="25" t="inlineStr">
         <is>
           <t>•  Podcast platforms return one row per episode. Streaming platforms handle both movies and series, with flexible season picks (all · 1-3 · 1,4,6).</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="23" t="inlineStr">
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="24" t="inlineStr">
         <is>
           <t>•  SiriusXM title search is Netflix-style: one device code the first time on a new computer, then automatic. Pasting a SiriusXM show link never needs a login.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="24" t="inlineStr">
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="25" t="inlineStr">
         <is>
           <t>•  Audible returns TWO rows per audiobook — the direct audible.com/pd listen link AND the parallel amazon.com/dp 'Audible Audio Edition' (a different ASIN) — each labeled Audible / Amazon in the PLATFORM column.</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="23" t="inlineStr">
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="24" t="inlineStr">
         <is>
           <t>•  Amazon captures every clickstream form — all offer ASINs, the GTI in both encodings, shells + episodes, every film edition, and Amazon Channels (Lionsgate+, Starz…).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="17">
     <mergeCell ref="A32:G32"/>
     <mergeCell ref="A36:G36"/>
     <mergeCell ref="A33:G33"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A40:G40"/>
     <mergeCell ref="A31:G31"/>
     <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A39:G39"/>
     <mergeCell ref="A34:G34"/>
     <mergeCell ref="A35:G35"/>
     <mergeCell ref="A26:G26"/>
-    <mergeCell ref="A30:G30"/>
+    <mergeCell ref="A38:G38"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A28:G28"/>
     <mergeCell ref="A19:G19"/>
     <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A37:G37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Coverage Excel: add Games (gametool_content) companion row
Adds a visible Games companion section/row to StreamScout-Platforms.xlsx so
gametool_content shows up in the grid, not just the footnotes.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/streamscout/StreamScout-Platforms.xlsx
+++ b/streamscout/StreamScout-Platforms.xlsx
@@ -660,7 +660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4.5" customWidth="1" min="1" max="1"/>
@@ -682,7 +682,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  One tool → every watch / play id  ·  21 platforms  ·  movies, series, podcasts, audiobooks &amp; books</t>
+          <t xml:space="preserve">  One tool → every watch / play id  ·  21 platforms + games companion  ·  movies, series, podcasts, audiobooks, books &amp; games</t>
         </is>
       </c>
     </row>
@@ -1507,92 +1507,137 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="26" customHeight="1">
-      <c r="A31" s="23" t="inlineStr">
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>🎮  Games companion  ·  1   (gametool_content — buy · play, feeds the content map)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="21" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Games</t>
+        </is>
+      </c>
+      <c r="C31" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D31" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>No login</t>
+        </is>
+      </c>
+      <c r="F31" s="11" t="inlineStr">
+        <is>
+          <t>buy + play links · 19 stores</t>
+        </is>
+      </c>
+      <c r="G31" s="12" t="inlineStr">
+        <is>
+          <t>streamscout/gametool_content — every buy/play URL across Steam, Epic, GOG, Nintendo, PlayStation, Xbox, Apple, Google Play, Battle.net (live) + Amazon/Luna/Best Buy/GameStop/Walmart/Target/Eneba/Loaded/G2A. Content-map terms; sibling gametool_hostmap emits the hostmap form.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="26" customHeight="1">
+      <c r="A33" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  Good to know</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="24" t="inlineStr">
-        <is>
-          <t>•  16 of 21 platforms need NO login. Only 5 need anything: Netflix &amp; HBO Max (browser login), Spotify (free API key), and Disney+ &amp; SiriusXM (situational).</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="25" t="inlineStr">
-        <is>
-          <t>•  Access legend:  No login = anonymous  ·  Browser login = a Firefox/Chromium window drives itself  ·  Free API key = Spotify Client ID+Secret  ·  Situational = usually none, occasional login.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="24" t="inlineStr">
         <is>
-          <t>•  Every run writes one CSV to your Desktop:  SHOW · URL · PRODUCTION · PLATFORM · SEASON.  PRODUCTION (studio) fills in automatically; SEASON is blank for movies, podcasts &amp; audiobooks (and Apple TV+, BritBox &amp; YouTube), and carries Book N for a book franchise.</t>
+          <t>•  16 of 21 platforms need NO login. Only 5 need anything: Netflix &amp; HBO Max (browser login), Spotify (free API key), and Disney+ &amp; SiriusXM (situational).</t>
         </is>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="25" t="inlineStr">
         <is>
-          <t>•  Books resolves a whole franchise to ONE show: purchase (Amazon Kindle/Print, Bookshop, Costco…), audiobook (Audible, Apple, Amazon), and LIBRARY holds (Libby/OverDrive) — with content-map retail proxies for the bot-walled stores. Its URLs feed the CONTENT map, so slugs keep their punctuation (p/merciless-saints).</t>
+          <t>•  Access legend:  No login = anonymous  ·  Browser login = a Firefox/Chromium window drives itself  ·  Free API key = Spotify Client ID+Secret  ·  Situational = usually none, occasional login.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="24" t="inlineStr">
         <is>
-          <t>•  Companion resolver: gametool_content (in streamscout/gametool_content) does the same job for VIDEO GAMES — every buy/play URL across 19 stores, also as content-map terms. Its sibling gametool_hostmap emits the punctuation-stripped hostmap form for a different pipeline.</t>
+          <t>•  Every run writes one CSV to your Desktop:  SHOW · URL · PRODUCTION · PLATFORM · SEASON.  PRODUCTION (studio) fills in automatically; SEASON is blank for movies, podcasts &amp; audiobooks (and Apple TV+, BritBox &amp; YouTube), and carries Book N for a book franchise.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="25" t="inlineStr">
         <is>
-          <t>•  Podcast platforms return one row per episode. Streaming platforms handle both movies and series, with flexible season picks (all · 1-3 · 1,4,6).</t>
+          <t>•  Books resolves a whole franchise to ONE show: purchase (Amazon Kindle/Print, Bookshop, Costco…), audiobook (Audible, Apple, Amazon), and LIBRARY holds (Libby/OverDrive) — with content-map retail proxies for the bot-walled stores. Its URLs feed the CONTENT map, so slugs keep their punctuation (p/merciless-saints).</t>
         </is>
       </c>
     </row>
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="24" t="inlineStr">
         <is>
-          <t>•  SiriusXM title search is Netflix-style: one device code the first time on a new computer, then automatic. Pasting a SiriusXM show link never needs a login.</t>
+          <t>•  Companion resolver: gametool_content (in streamscout/gametool_content) does the same job for VIDEO GAMES — every buy/play URL across 19 stores, also as content-map terms. Its sibling gametool_hostmap emits the punctuation-stripped hostmap form for a different pipeline.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="25" t="inlineStr">
         <is>
-          <t>•  Audible returns TWO rows per audiobook — the direct audible.com/pd listen link AND the parallel amazon.com/dp 'Audible Audio Edition' (a different ASIN) — each labeled Audible / Amazon in the PLATFORM column.</t>
+          <t>•  Podcast platforms return one row per episode. Streaming platforms handle both movies and series, with flexible season picks (all · 1-3 · 1,4,6).</t>
         </is>
       </c>
     </row>
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="24" t="inlineStr">
         <is>
+          <t>•  SiriusXM title search is Netflix-style: one device code the first time on a new computer, then automatic. Pasting a SiriusXM show link never needs a login.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="25" t="inlineStr">
+        <is>
+          <t>•  Audible returns TWO rows per audiobook — the direct audible.com/pd listen link AND the parallel amazon.com/dp 'Audible Audio Edition' (a different ASIN) — each labeled Audible / Amazon in the PLATFORM column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="24" t="inlineStr">
+        <is>
           <t>•  Amazon captures every clickstream form — all offer ASINs, the GTI in both encodings, shells + episodes, every film edition, and Amazon Channels (Lionsgate+, Starz…).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="A32:G32"/>
+  <mergeCells count="18">
     <mergeCell ref="A36:G36"/>
     <mergeCell ref="A33:G33"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A40:G40"/>
-    <mergeCell ref="A31:G31"/>
     <mergeCell ref="A3:G3"/>
     <mergeCell ref="A39:G39"/>
     <mergeCell ref="A34:G34"/>
     <mergeCell ref="A35:G35"/>
     <mergeCell ref="A26:G26"/>
+    <mergeCell ref="A30:G30"/>
+    <mergeCell ref="A2:G2"/>
     <mergeCell ref="A38:G38"/>
-    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A42:G42"/>
     <mergeCell ref="A28:G28"/>
+    <mergeCell ref="A41:G41"/>
     <mergeCell ref="A19:G19"/>
     <mergeCell ref="A5:G5"/>
     <mergeCell ref="A37:G37"/>

</xml_diff>

<commit_message>
Coverage Excel: add Games (gametool_content) companion row (#192)
Adds a visible Games companion section/row to StreamScout-Platforms.xlsx so
gametool_content shows up in the grid, not just the footnotes.

Co-authored-by: Jessie <jessie@Trina-McGillicutty.local>
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/streamscout/StreamScout-Platforms.xlsx
+++ b/streamscout/StreamScout-Platforms.xlsx
@@ -660,7 +660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4.5" customWidth="1" min="1" max="1"/>
@@ -682,7 +682,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  One tool → every watch / play id  ·  21 platforms  ·  movies, series, podcasts, audiobooks &amp; books</t>
+          <t xml:space="preserve">  One tool → every watch / play id  ·  21 platforms + games companion  ·  movies, series, podcasts, audiobooks, books &amp; games</t>
         </is>
       </c>
     </row>
@@ -1507,92 +1507,137 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="26" customHeight="1">
-      <c r="A31" s="23" t="inlineStr">
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>🎮  Games companion  ·  1   (gametool_content — buy · play, feeds the content map)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="21" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Games</t>
+        </is>
+      </c>
+      <c r="C31" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D31" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>No login</t>
+        </is>
+      </c>
+      <c r="F31" s="11" t="inlineStr">
+        <is>
+          <t>buy + play links · 19 stores</t>
+        </is>
+      </c>
+      <c r="G31" s="12" t="inlineStr">
+        <is>
+          <t>streamscout/gametool_content — every buy/play URL across Steam, Epic, GOG, Nintendo, PlayStation, Xbox, Apple, Google Play, Battle.net (live) + Amazon/Luna/Best Buy/GameStop/Walmart/Target/Eneba/Loaded/G2A. Content-map terms; sibling gametool_hostmap emits the hostmap form.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="26" customHeight="1">
+      <c r="A33" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  Good to know</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="24" t="inlineStr">
-        <is>
-          <t>•  16 of 21 platforms need NO login. Only 5 need anything: Netflix &amp; HBO Max (browser login), Spotify (free API key), and Disney+ &amp; SiriusXM (situational).</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="25" t="inlineStr">
-        <is>
-          <t>•  Access legend:  No login = anonymous  ·  Browser login = a Firefox/Chromium window drives itself  ·  Free API key = Spotify Client ID+Secret  ·  Situational = usually none, occasional login.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="24" t="inlineStr">
         <is>
-          <t>•  Every run writes one CSV to your Desktop:  SHOW · URL · PRODUCTION · PLATFORM · SEASON.  PRODUCTION (studio) fills in automatically; SEASON is blank for movies, podcasts &amp; audiobooks (and Apple TV+, BritBox &amp; YouTube), and carries Book N for a book franchise.</t>
+          <t>•  16 of 21 platforms need NO login. Only 5 need anything: Netflix &amp; HBO Max (browser login), Spotify (free API key), and Disney+ &amp; SiriusXM (situational).</t>
         </is>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="25" t="inlineStr">
         <is>
-          <t>•  Books resolves a whole franchise to ONE show: purchase (Amazon Kindle/Print, Bookshop, Costco…), audiobook (Audible, Apple, Amazon), and LIBRARY holds (Libby/OverDrive) — with content-map retail proxies for the bot-walled stores. Its URLs feed the CONTENT map, so slugs keep their punctuation (p/merciless-saints).</t>
+          <t>•  Access legend:  No login = anonymous  ·  Browser login = a Firefox/Chromium window drives itself  ·  Free API key = Spotify Client ID+Secret  ·  Situational = usually none, occasional login.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="24" t="inlineStr">
         <is>
-          <t>•  Companion resolver: gametool_content (in streamscout/gametool_content) does the same job for VIDEO GAMES — every buy/play URL across 19 stores, also as content-map terms. Its sibling gametool_hostmap emits the punctuation-stripped hostmap form for a different pipeline.</t>
+          <t>•  Every run writes one CSV to your Desktop:  SHOW · URL · PRODUCTION · PLATFORM · SEASON.  PRODUCTION (studio) fills in automatically; SEASON is blank for movies, podcasts &amp; audiobooks (and Apple TV+, BritBox &amp; YouTube), and carries Book N for a book franchise.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="25" t="inlineStr">
         <is>
-          <t>•  Podcast platforms return one row per episode. Streaming platforms handle both movies and series, with flexible season picks (all · 1-3 · 1,4,6).</t>
+          <t>•  Books resolves a whole franchise to ONE show: purchase (Amazon Kindle/Print, Bookshop, Costco…), audiobook (Audible, Apple, Amazon), and LIBRARY holds (Libby/OverDrive) — with content-map retail proxies for the bot-walled stores. Its URLs feed the CONTENT map, so slugs keep their punctuation (p/merciless-saints).</t>
         </is>
       </c>
     </row>
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="24" t="inlineStr">
         <is>
-          <t>•  SiriusXM title search is Netflix-style: one device code the first time on a new computer, then automatic. Pasting a SiriusXM show link never needs a login.</t>
+          <t>•  Companion resolver: gametool_content (in streamscout/gametool_content) does the same job for VIDEO GAMES — every buy/play URL across 19 stores, also as content-map terms. Its sibling gametool_hostmap emits the punctuation-stripped hostmap form for a different pipeline.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="25" t="inlineStr">
         <is>
-          <t>•  Audible returns TWO rows per audiobook — the direct audible.com/pd listen link AND the parallel amazon.com/dp 'Audible Audio Edition' (a different ASIN) — each labeled Audible / Amazon in the PLATFORM column.</t>
+          <t>•  Podcast platforms return one row per episode. Streaming platforms handle both movies and series, with flexible season picks (all · 1-3 · 1,4,6).</t>
         </is>
       </c>
     </row>
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="24" t="inlineStr">
         <is>
+          <t>•  SiriusXM title search is Netflix-style: one device code the first time on a new computer, then automatic. Pasting a SiriusXM show link never needs a login.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="25" t="inlineStr">
+        <is>
+          <t>•  Audible returns TWO rows per audiobook — the direct audible.com/pd listen link AND the parallel amazon.com/dp 'Audible Audio Edition' (a different ASIN) — each labeled Audible / Amazon in the PLATFORM column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="24" t="inlineStr">
+        <is>
           <t>•  Amazon captures every clickstream form — all offer ASINs, the GTI in both encodings, shells + episodes, every film edition, and Amazon Channels (Lionsgate+, Starz…).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="A32:G32"/>
+  <mergeCells count="18">
     <mergeCell ref="A36:G36"/>
     <mergeCell ref="A33:G33"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A40:G40"/>
-    <mergeCell ref="A31:G31"/>
     <mergeCell ref="A3:G3"/>
     <mergeCell ref="A39:G39"/>
     <mergeCell ref="A34:G34"/>
     <mergeCell ref="A35:G35"/>
     <mergeCell ref="A26:G26"/>
+    <mergeCell ref="A30:G30"/>
+    <mergeCell ref="A2:G2"/>
     <mergeCell ref="A38:G38"/>
-    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A42:G42"/>
     <mergeCell ref="A28:G28"/>
+    <mergeCell ref="A41:G41"/>
     <mergeCell ref="A19:G19"/>
     <mergeCell ref="A5:G5"/>
     <mergeCell ref="A37:G37"/>

</xml_diff>

<commit_message>
StreamScout #22 Games: gametool_content as a first-class menu platform
- Add games_identifier.py: thin adapter wrapping streamscout/gametool_content
  so a Games menu pick runs the live multi-store search and returns rows in
  StreamScout schema (identifier = content-map term, platform = store).
- Register games in RESOLVER_PLATFORMS / RESOLVER_MODULE / URL_HINT_RESOLVERS /
  PLATFORM_ORDER (+ menu tag + dispatch print). SHOW = franchise on every row.
- Docs: coverage Excel/MD + Jenna how-to now list Games as platform #22
  (no-login 17 of 22).

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/streamscout/StreamScout-Platforms.xlsx
+++ b/streamscout/StreamScout-Platforms.xlsx
@@ -682,7 +682,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  One tool → every watch / play id  ·  21 platforms + games companion  ·  movies, series, podcasts, audiobooks, books &amp; games</t>
+          <t xml:space="preserve">  One tool → every watch / play id  ·  22 platforms  ·  movies, series, podcasts, audiobooks, books &amp; games</t>
         </is>
       </c>
     </row>
@@ -1510,7 +1510,7 @@
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>🎮  Games companion  ·  1   (gametool_content — buy · play, feeds the content map)</t>
+          <t>🎮  Games  ·  1   (buy · play — feeds the content map)</t>
         </is>
       </c>
     </row>
@@ -1547,7 +1547,7 @@
       </c>
       <c r="G31" s="12" t="inlineStr">
         <is>
-          <t>streamscout/gametool_content — every buy/play URL across Steam, Epic, GOG, Nintendo, PlayStation, Xbox, Apple, Google Play, Battle.net (live) + Amazon/Luna/Best Buy/GameStop/Walmart/Target/Eneba/Loaded/G2A. Content-map terms; sibling gametool_hostmap emits the hostmap form.</t>
+          <t>Menu pick like any other platform. Every buy/play URL across Steam, Epic, GOG, Nintendo, PlayStation, Xbox, Apple, Google Play, Battle.net (live) + Amazon/Luna/Best Buy/GameStop/Walmart/Target/Eneba/Loaded/G2A. Engine: streamscout/gametool_content; content-map terms; sibling gametool_hostmap emits the hostmap form.</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1561,7 @@
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="24" t="inlineStr">
         <is>
-          <t>•  16 of 21 platforms need NO login. Only 5 need anything: Netflix &amp; HBO Max (browser login), Spotify (free API key), and Disney+ &amp; SiriusXM (situational).</t>
+          <t>•  17 of 22 platforms need NO login. Only 5 need anything: Netflix &amp; HBO Max (browser login), Spotify (free API key), and Disney+ &amp; SiriusXM (situational).</t>
         </is>
       </c>
     </row>
@@ -1589,7 +1589,7 @@
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="24" t="inlineStr">
         <is>
-          <t>•  Companion resolver: gametool_content (in streamscout/gametool_content) does the same job for VIDEO GAMES — every buy/play URL across 19 stores, also as content-map terms. Its sibling gametool_hostmap emits the punctuation-stripped hostmap form for a different pipeline.</t>
+          <t>•  Games works like any other platform: pick Games, type a title/franchise, and get every buy/play URL across 19 stores as content-map terms (SHOW = the franchise on every row). Engine lives in streamscout/gametool_content; its sibling gametool_hostmap emits the punctuation-stripped hostmap form for a different pipeline.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
StreamScout #22 Games: gametool_content as a first-class menu platform (#193)
- Add games_identifier.py: thin adapter wrapping streamscout/gametool_content
  so a Games menu pick runs the live multi-store search and returns rows in
  StreamScout schema (identifier = content-map term, platform = store).
- Register games in RESOLVER_PLATFORMS / RESOLVER_MODULE / URL_HINT_RESOLVERS /
  PLATFORM_ORDER (+ menu tag + dispatch print). SHOW = franchise on every row.
- Docs: coverage Excel/MD + Jenna how-to now list Games as platform #22
  (no-login 17 of 22).

Co-authored-by: Jessie <jessie@Trina-McGillicutty.local>
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/streamscout/StreamScout-Platforms.xlsx
+++ b/streamscout/StreamScout-Platforms.xlsx
@@ -682,7 +682,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  One tool → every watch / play id  ·  21 platforms + games companion  ·  movies, series, podcasts, audiobooks, books &amp; games</t>
+          <t xml:space="preserve">  One tool → every watch / play id  ·  22 platforms  ·  movies, series, podcasts, audiobooks, books &amp; games</t>
         </is>
       </c>
     </row>
@@ -1510,7 +1510,7 @@
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>🎮  Games companion  ·  1   (gametool_content — buy · play, feeds the content map)</t>
+          <t>🎮  Games  ·  1   (buy · play — feeds the content map)</t>
         </is>
       </c>
     </row>
@@ -1547,7 +1547,7 @@
       </c>
       <c r="G31" s="12" t="inlineStr">
         <is>
-          <t>streamscout/gametool_content — every buy/play URL across Steam, Epic, GOG, Nintendo, PlayStation, Xbox, Apple, Google Play, Battle.net (live) + Amazon/Luna/Best Buy/GameStop/Walmart/Target/Eneba/Loaded/G2A. Content-map terms; sibling gametool_hostmap emits the hostmap form.</t>
+          <t>Menu pick like any other platform. Every buy/play URL across Steam, Epic, GOG, Nintendo, PlayStation, Xbox, Apple, Google Play, Battle.net (live) + Amazon/Luna/Best Buy/GameStop/Walmart/Target/Eneba/Loaded/G2A. Engine: streamscout/gametool_content; content-map terms; sibling gametool_hostmap emits the hostmap form.</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1561,7 @@
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="24" t="inlineStr">
         <is>
-          <t>•  16 of 21 platforms need NO login. Only 5 need anything: Netflix &amp; HBO Max (browser login), Spotify (free API key), and Disney+ &amp; SiriusXM (situational).</t>
+          <t>•  17 of 22 platforms need NO login. Only 5 need anything: Netflix &amp; HBO Max (browser login), Spotify (free API key), and Disney+ &amp; SiriusXM (situational).</t>
         </is>
       </c>
     </row>
@@ -1589,7 +1589,7 @@
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="24" t="inlineStr">
         <is>
-          <t>•  Companion resolver: gametool_content (in streamscout/gametool_content) does the same job for VIDEO GAMES — every buy/play URL across 19 stores, also as content-map terms. Its sibling gametool_hostmap emits the punctuation-stripped hostmap form for a different pipeline.</t>
+          <t>•  Games works like any other platform: pick Games, type a title/franchise, and get every buy/play URL across 19 stores as content-map terms (SHOW = the franchise on every row). Engine lives in streamscout/gametool_content; its sibling gametool_hostmap emits the punctuation-stripped hostmap form for a different pipeline.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
StreamScout: Jenna/Promy package — explicit how-to MD + refreshed 23-platform xlsx
- StreamScout-HowTo-Jenna-Explicit.md: step-by-step Promy integration guide —
  the streamscout_query() entry point and every parameter, platform groups,
  podcasts = native audio + NPR + YouTube, and the two new YouTube client
  choices (include_clips + the fair-survey limit) with worked numbers and a
  suggested Promy prompt.
- build_platforms_xlsx.py: add NPR to the podcasts section, refresh the YouTube
  note (full-vs-clips + fair-survey cap), update the no-login count (18) and add
  good-to-know bullets for the podcast+YouTube sweep and the YouTube knobs.
- Regenerated StreamScout-Platforms.xlsx (now 23 platforms).

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/streamscout/StreamScout-Platforms.xlsx
+++ b/streamscout/StreamScout-Platforms.xlsx
@@ -289,10 +289,10 @@
     <xf numFmtId="0" fontId="17" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
@@ -660,7 +660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4.5" customWidth="1" min="1" max="1"/>
@@ -682,7 +682,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  One tool → every watch / play id  ·  22 platforms  ·  movies, series, podcasts, audiobooks, books &amp; games</t>
+          <t xml:space="preserve">  One tool → every watch / play id  ·  23 platforms  ·  movies, series, podcasts, audiobooks, books &amp; games</t>
         </is>
       </c>
     </row>
@@ -1194,14 +1194,14 @@
       </c>
       <c r="G18" s="12" t="inlineStr">
         <is>
-          <t>Channel Videos tab; Shorts excluded</t>
+          <t>Full videos (Videos tab) by default; opt-in clips (Shorts); fair-survey cap 600 across the timespan</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>🎧  Podcasts  ·  6</t>
+          <t>🎧  Podcasts  ·  7</t>
         </is>
       </c>
     </row>
@@ -1419,228 +1419,281 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="6" t="inlineStr">
+    <row r="26" ht="21" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>NPR</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>No login</t>
+        </is>
+      </c>
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>every episode npr.org URL</t>
+        </is>
+      </c>
+      <c r="G26" s="12" t="inlineStr">
+        <is>
+          <t>Reads the show's public feed; one row per episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t>📚  Audiobooks  ·  1</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="21" customHeight="1">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>▸</t>
-        </is>
-      </c>
-      <c r="B27" s="8" t="inlineStr">
+    <row r="28" ht="21" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>Audible</t>
         </is>
       </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E27" s="10" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E28" s="10" t="inlineStr">
         <is>
           <t>No login</t>
         </is>
       </c>
-      <c r="F27" s="11" t="inlineStr">
+      <c r="F28" s="11" t="inlineStr">
         <is>
           <t>direct Audible + via-Amazon</t>
         </is>
       </c>
-      <c r="G27" s="12" t="inlineStr">
+      <c r="G28" s="12" t="inlineStr">
         <is>
           <t>TWO rows / title: audible.com/pd + amazon.com/dp (different ASINs)</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="6" t="inlineStr">
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t>📖  Books  ·  1   (buy · listen · library — feeds the content map)</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="21" customHeight="1">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>▸</t>
-        </is>
-      </c>
-      <c r="B29" s="8" t="inlineStr">
+    <row r="30" ht="21" customHeight="1">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>Books</t>
         </is>
       </c>
-      <c r="C29" s="22" t="inlineStr">
+      <c r="C30" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D29" s="22" t="inlineStr">
+      <c r="D30" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E29" s="10" t="inlineStr">
+      <c r="E30" s="10" t="inlineStr">
         <is>
           <t>No login</t>
         </is>
       </c>
-      <c r="F29" s="11" t="inlineStr">
+      <c r="F30" s="11" t="inlineStr">
         <is>
           <t>buy + listen + library links</t>
         </is>
       </c>
-      <c r="G29" s="12" t="inlineStr">
+      <c r="G30" s="12" t="inlineStr">
         <is>
           <t>Whole franchise → ONE show, SEASON = Book N. Amazon Kindle/Print/Audio, Audible, Apple Books, Libby holds, + retail proxies (Target/BAM, Walmart, B&amp;N, Bookshop, Costco). Feeds the CONTENT map (punctuation kept).</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="6" t="inlineStr">
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="6" t="inlineStr">
         <is>
           <t>🎮  Games  ·  1   (buy · play — feeds the content map)</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="21" customHeight="1">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>▸</t>
-        </is>
-      </c>
-      <c r="B31" s="8" t="inlineStr">
+    <row r="32" ht="21" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>Games</t>
         </is>
       </c>
-      <c r="C31" s="22" t="inlineStr">
+      <c r="C32" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D31" s="22" t="inlineStr">
+      <c r="D32" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E31" s="10" t="inlineStr">
+      <c r="E32" s="10" t="inlineStr">
         <is>
           <t>No login</t>
         </is>
       </c>
-      <c r="F31" s="11" t="inlineStr">
+      <c r="F32" s="11" t="inlineStr">
         <is>
           <t>buy + play links · 19 stores</t>
         </is>
       </c>
-      <c r="G31" s="12" t="inlineStr">
+      <c r="G32" s="12" t="inlineStr">
         <is>
           <t>Menu pick like any other platform. Every buy/play URL across Steam, Epic, GOG, Nintendo, PlayStation, Xbox, Apple, Google Play, Battle.net (live) + Amazon/Luna/Best Buy/GameStop/Walmart/Target/Eneba/Loaded/G2A. Engine: streamscout/gametool_content; content-map terms; sibling gametool_hostmap emits the hostmap form.</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="26" customHeight="1">
-      <c r="A33" s="23" t="inlineStr">
+    <row r="34" ht="26" customHeight="1">
+      <c r="A34" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  Good to know</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="24" t="inlineStr">
-        <is>
-          <t>•  17 of 22 platforms need NO login. Only 5 need anything: Netflix &amp; HBO Max (browser login), Spotify (free API key), and Disney+ &amp; SiriusXM (situational).</t>
-        </is>
-      </c>
-    </row>
     <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="25" t="inlineStr">
+      <c r="A35" s="24" t="inlineStr">
+        <is>
+          <t>•  18 of 23 platforms need NO login. Only 5 need anything: Netflix &amp; HBO Max (browser login), Spotify (free API key), and Disney+ &amp; SiriusXM (situational).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="25" t="inlineStr">
+        <is>
+          <t>•  A PODCAST query sweeps the native audio platforms (Spotify, Apple Podcasts, iHeart, Pandora, Amazon Podcasts, SiriusXM, NPR) AND the show's YouTube channel in one go — listeners + video viewers together.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="24" t="inlineStr">
+        <is>
+          <t>•  YouTube, full-vs-clips (client choice in Promy): FULL episodes/videos only (the long-form Videos tab) is the default; INCLUDE CLIPS also folds in Shorts. A fair-survey cap (default 600) even-strides a big channel down across its whole timespan — a representative spread, not just the most recent block (0 = no cap).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="25" t="inlineStr">
         <is>
           <t>•  Access legend:  No login = anonymous  ·  Browser login = a Firefox/Chromium window drives itself  ·  Free API key = Spotify Client ID+Secret  ·  Situational = usually none, occasional login.</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="24" t="inlineStr">
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="24" t="inlineStr">
         <is>
           <t>•  Every run writes one CSV to your Desktop:  SHOW · URL · PRODUCTION · PLATFORM · SEASON.  PRODUCTION (studio) fills in automatically; SEASON is blank for movies, podcasts &amp; audiobooks (and Apple TV+, BritBox &amp; YouTube), and carries Book N for a book franchise.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="25" t="inlineStr">
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="25" t="inlineStr">
         <is>
           <t>•  Books resolves a whole franchise to ONE show: purchase (Amazon Kindle/Print, Bookshop, Costco…), audiobook (Audible, Apple, Amazon), and LIBRARY holds (Libby/OverDrive) — with content-map retail proxies for the bot-walled stores. Its URLs feed the CONTENT map, so slugs keep their punctuation (p/merciless-saints).</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="24" t="inlineStr">
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="24" t="inlineStr">
         <is>
           <t>•  Games works like any other platform: pick Games, type a title/franchise, and get every buy/play URL across 19 stores as content-map terms (SHOW = the franchise on every row). Engine lives in streamscout/gametool_content; its sibling gametool_hostmap emits the punctuation-stripped hostmap form for a different pipeline.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="25" t="inlineStr">
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="25" t="inlineStr">
         <is>
           <t>•  Podcast platforms return one row per episode. Streaming platforms handle both movies and series, with flexible season picks (all · 1-3 · 1,4,6).</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="24" t="inlineStr">
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="24" t="inlineStr">
         <is>
           <t>•  SiriusXM title search is Netflix-style: one device code the first time on a new computer, then automatic. Pasting a SiriusXM show link never needs a login.</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="25" t="inlineStr">
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="25" t="inlineStr">
         <is>
           <t>•  Audible returns TWO rows per audiobook — the direct audible.com/pd listen link AND the parallel amazon.com/dp 'Audible Audio Edition' (a different ASIN) — each labeled Audible / Amazon in the PLATFORM column.</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="30" customHeight="1">
-      <c r="A42" s="24" t="inlineStr">
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="24" t="inlineStr">
         <is>
           <t>•  Amazon captures every clickstream form — all offer ASINs, the GTI in both encodings, shells + episodes, every film edition, and Amazon Channels (Lionsgate+, Starz…).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="A36:G36"/>
-    <mergeCell ref="A33:G33"/>
-    <mergeCell ref="A1:G1"/>
+  <mergeCells count="20">
+    <mergeCell ref="A35:G35"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A38:G38"/>
+    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A43:G43"/>
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A44:G44"/>
     <mergeCell ref="A40:G40"/>
-    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A31:G31"/>
     <mergeCell ref="A39:G39"/>
     <mergeCell ref="A34:G34"/>
-    <mergeCell ref="A35:G35"/>
-    <mergeCell ref="A26:G26"/>
-    <mergeCell ref="A30:G30"/>
+    <mergeCell ref="A45:G45"/>
+    <mergeCell ref="A36:G36"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A41:G41"/>
+    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="A27:G27"/>
+    <mergeCell ref="A3:G3"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A38:G38"/>
     <mergeCell ref="A42:G42"/>
-    <mergeCell ref="A28:G28"/>
-    <mergeCell ref="A41:G41"/>
-    <mergeCell ref="A19:G19"/>
-    <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A37:G37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
StreamScout: Jenna/Promy package — explicit how-to MD + refreshed 23-platform xlsx (#311)
- StreamScout-HowTo-Jenna-Explicit.md: step-by-step Promy integration guide —
  the streamscout_query() entry point and every parameter, platform groups,
  podcasts = native audio + NPR + YouTube, and the two new YouTube client
  choices (include_clips + the fair-survey limit) with worked numbers and a
  suggested Promy prompt.
- build_platforms_xlsx.py: add NPR to the podcasts section, refresh the YouTube
  note (full-vs-clips + fair-survey cap), update the no-login count (18) and add
  good-to-know bullets for the podcast+YouTube sweep and the YouTube knobs.
- Regenerated StreamScout-Platforms.xlsx (now 23 platforms).

Co-authored-by: Jessie <jessie@Trina-McGillicutty.local>
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/streamscout/StreamScout-Platforms.xlsx
+++ b/streamscout/StreamScout-Platforms.xlsx
@@ -289,10 +289,10 @@
     <xf numFmtId="0" fontId="17" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
@@ -660,7 +660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4.5" customWidth="1" min="1" max="1"/>
@@ -682,7 +682,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  One tool → every watch / play id  ·  22 platforms  ·  movies, series, podcasts, audiobooks, books &amp; games</t>
+          <t xml:space="preserve">  One tool → every watch / play id  ·  23 platforms  ·  movies, series, podcasts, audiobooks, books &amp; games</t>
         </is>
       </c>
     </row>
@@ -1194,14 +1194,14 @@
       </c>
       <c r="G18" s="12" t="inlineStr">
         <is>
-          <t>Channel Videos tab; Shorts excluded</t>
+          <t>Full videos (Videos tab) by default; opt-in clips (Shorts); fair-survey cap 600 across the timespan</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>🎧  Podcasts  ·  6</t>
+          <t>🎧  Podcasts  ·  7</t>
         </is>
       </c>
     </row>
@@ -1419,228 +1419,281 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="6" t="inlineStr">
+    <row r="26" ht="21" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>NPR</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>No login</t>
+        </is>
+      </c>
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>every episode npr.org URL</t>
+        </is>
+      </c>
+      <c r="G26" s="12" t="inlineStr">
+        <is>
+          <t>Reads the show's public feed; one row per episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t>📚  Audiobooks  ·  1</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="21" customHeight="1">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>▸</t>
-        </is>
-      </c>
-      <c r="B27" s="8" t="inlineStr">
+    <row r="28" ht="21" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>Audible</t>
         </is>
       </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E27" s="10" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E28" s="10" t="inlineStr">
         <is>
           <t>No login</t>
         </is>
       </c>
-      <c r="F27" s="11" t="inlineStr">
+      <c r="F28" s="11" t="inlineStr">
         <is>
           <t>direct Audible + via-Amazon</t>
         </is>
       </c>
-      <c r="G27" s="12" t="inlineStr">
+      <c r="G28" s="12" t="inlineStr">
         <is>
           <t>TWO rows / title: audible.com/pd + amazon.com/dp (different ASINs)</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="6" t="inlineStr">
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t>📖  Books  ·  1   (buy · listen · library — feeds the content map)</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="21" customHeight="1">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>▸</t>
-        </is>
-      </c>
-      <c r="B29" s="8" t="inlineStr">
+    <row r="30" ht="21" customHeight="1">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>Books</t>
         </is>
       </c>
-      <c r="C29" s="22" t="inlineStr">
+      <c r="C30" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D29" s="22" t="inlineStr">
+      <c r="D30" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E29" s="10" t="inlineStr">
+      <c r="E30" s="10" t="inlineStr">
         <is>
           <t>No login</t>
         </is>
       </c>
-      <c r="F29" s="11" t="inlineStr">
+      <c r="F30" s="11" t="inlineStr">
         <is>
           <t>buy + listen + library links</t>
         </is>
       </c>
-      <c r="G29" s="12" t="inlineStr">
+      <c r="G30" s="12" t="inlineStr">
         <is>
           <t>Whole franchise → ONE show, SEASON = Book N. Amazon Kindle/Print/Audio, Audible, Apple Books, Libby holds, + retail proxies (Target/BAM, Walmart, B&amp;N, Bookshop, Costco). Feeds the CONTENT map (punctuation kept).</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="6" t="inlineStr">
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="6" t="inlineStr">
         <is>
           <t>🎮  Games  ·  1   (buy · play — feeds the content map)</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="21" customHeight="1">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>▸</t>
-        </is>
-      </c>
-      <c r="B31" s="8" t="inlineStr">
+    <row r="32" ht="21" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>Games</t>
         </is>
       </c>
-      <c r="C31" s="22" t="inlineStr">
+      <c r="C32" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D31" s="22" t="inlineStr">
+      <c r="D32" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E31" s="10" t="inlineStr">
+      <c r="E32" s="10" t="inlineStr">
         <is>
           <t>No login</t>
         </is>
       </c>
-      <c r="F31" s="11" t="inlineStr">
+      <c r="F32" s="11" t="inlineStr">
         <is>
           <t>buy + play links · 19 stores</t>
         </is>
       </c>
-      <c r="G31" s="12" t="inlineStr">
+      <c r="G32" s="12" t="inlineStr">
         <is>
           <t>Menu pick like any other platform. Every buy/play URL across Steam, Epic, GOG, Nintendo, PlayStation, Xbox, Apple, Google Play, Battle.net (live) + Amazon/Luna/Best Buy/GameStop/Walmart/Target/Eneba/Loaded/G2A. Engine: streamscout/gametool_content; content-map terms; sibling gametool_hostmap emits the hostmap form.</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="26" customHeight="1">
-      <c r="A33" s="23" t="inlineStr">
+    <row r="34" ht="26" customHeight="1">
+      <c r="A34" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  Good to know</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="24" t="inlineStr">
-        <is>
-          <t>•  17 of 22 platforms need NO login. Only 5 need anything: Netflix &amp; HBO Max (browser login), Spotify (free API key), and Disney+ &amp; SiriusXM (situational).</t>
-        </is>
-      </c>
-    </row>
     <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="25" t="inlineStr">
+      <c r="A35" s="24" t="inlineStr">
+        <is>
+          <t>•  18 of 23 platforms need NO login. Only 5 need anything: Netflix &amp; HBO Max (browser login), Spotify (free API key), and Disney+ &amp; SiriusXM (situational).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="25" t="inlineStr">
+        <is>
+          <t>•  A PODCAST query sweeps the native audio platforms (Spotify, Apple Podcasts, iHeart, Pandora, Amazon Podcasts, SiriusXM, NPR) AND the show's YouTube channel in one go — listeners + video viewers together.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="24" t="inlineStr">
+        <is>
+          <t>•  YouTube, full-vs-clips (client choice in Promy): FULL episodes/videos only (the long-form Videos tab) is the default; INCLUDE CLIPS also folds in Shorts. A fair-survey cap (default 600) even-strides a big channel down across its whole timespan — a representative spread, not just the most recent block (0 = no cap).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="25" t="inlineStr">
         <is>
           <t>•  Access legend:  No login = anonymous  ·  Browser login = a Firefox/Chromium window drives itself  ·  Free API key = Spotify Client ID+Secret  ·  Situational = usually none, occasional login.</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="24" t="inlineStr">
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="24" t="inlineStr">
         <is>
           <t>•  Every run writes one CSV to your Desktop:  SHOW · URL · PRODUCTION · PLATFORM · SEASON.  PRODUCTION (studio) fills in automatically; SEASON is blank for movies, podcasts &amp; audiobooks (and Apple TV+, BritBox &amp; YouTube), and carries Book N for a book franchise.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="25" t="inlineStr">
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="25" t="inlineStr">
         <is>
           <t>•  Books resolves a whole franchise to ONE show: purchase (Amazon Kindle/Print, Bookshop, Costco…), audiobook (Audible, Apple, Amazon), and LIBRARY holds (Libby/OverDrive) — with content-map retail proxies for the bot-walled stores. Its URLs feed the CONTENT map, so slugs keep their punctuation (p/merciless-saints).</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="24" t="inlineStr">
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="24" t="inlineStr">
         <is>
           <t>•  Games works like any other platform: pick Games, type a title/franchise, and get every buy/play URL across 19 stores as content-map terms (SHOW = the franchise on every row). Engine lives in streamscout/gametool_content; its sibling gametool_hostmap emits the punctuation-stripped hostmap form for a different pipeline.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="25" t="inlineStr">
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="25" t="inlineStr">
         <is>
           <t>•  Podcast platforms return one row per episode. Streaming platforms handle both movies and series, with flexible season picks (all · 1-3 · 1,4,6).</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="24" t="inlineStr">
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="24" t="inlineStr">
         <is>
           <t>•  SiriusXM title search is Netflix-style: one device code the first time on a new computer, then automatic. Pasting a SiriusXM show link never needs a login.</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="25" t="inlineStr">
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="25" t="inlineStr">
         <is>
           <t>•  Audible returns TWO rows per audiobook — the direct audible.com/pd listen link AND the parallel amazon.com/dp 'Audible Audio Edition' (a different ASIN) — each labeled Audible / Amazon in the PLATFORM column.</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="30" customHeight="1">
-      <c r="A42" s="24" t="inlineStr">
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="24" t="inlineStr">
         <is>
           <t>•  Amazon captures every clickstream form — all offer ASINs, the GTI in both encodings, shells + episodes, every film edition, and Amazon Channels (Lionsgate+, Starz…).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="A36:G36"/>
-    <mergeCell ref="A33:G33"/>
-    <mergeCell ref="A1:G1"/>
+  <mergeCells count="20">
+    <mergeCell ref="A35:G35"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A38:G38"/>
+    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A43:G43"/>
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A44:G44"/>
     <mergeCell ref="A40:G40"/>
-    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A31:G31"/>
     <mergeCell ref="A39:G39"/>
     <mergeCell ref="A34:G34"/>
-    <mergeCell ref="A35:G35"/>
-    <mergeCell ref="A26:G26"/>
-    <mergeCell ref="A30:G30"/>
+    <mergeCell ref="A45:G45"/>
+    <mergeCell ref="A36:G36"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A41:G41"/>
+    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="A27:G27"/>
+    <mergeCell ref="A3:G3"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A38:G38"/>
     <mergeCell ref="A42:G42"/>
-    <mergeCell ref="A28:G28"/>
-    <mergeCell ref="A41:G41"/>
-    <mergeCell ref="A19:G19"/>
-    <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A37:G37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>